<commit_message>
Add split 60 evaluation recap
</commit_message>
<xml_diff>
--- a/analysis_outputs/final_hyperparameter_summary.xlsx
+++ b/analysis_outputs/final_hyperparameter_summary.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final_Hyperparameters" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment_Grid" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final_Model_Metrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Split_Comparison" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -57,10 +60,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,265 +448,265 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>YOLOv12N</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Model dengan validation mAP50 tertinggi pada rekap final.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>split</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80:10:10</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Train:validation:test internal.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>epoch</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Epoch setting final.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>batch</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Batch size training.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>imgsz</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Ukuran input YOLO.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>optimizer</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>AdamW</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Optimizer training.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>lr0</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Initial learning rate.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>lrf</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Final learning-rate fraction.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>weight_decay</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Weight decay.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>mosaic</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Augmentasi mosaic.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>mixup</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Augmentasi mixup.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Seed split/training.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>patience</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Early-stopping patience.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>cos_lr</t>
         </is>
       </c>
-      <c r="B15" t="b">
+      <c r="B15" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Cosine LR schedule.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>workers</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Data loader workers.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>device</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Device training dari args.yaml.</t>
         </is>
@@ -727,246 +739,246 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="46" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Variants</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Epochs</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Batch</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Image_Size</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Optimizer</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>LR0</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>LRF</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Weight_Decay</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Mosaic</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Mixup</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Final comparison</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>80:10:10</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>YOLOv12N/S/M/L/X</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>50, 100</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>AdamW</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>validated + selected internal test</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Final comparison</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>70:15:15</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>YOLOv12N/S/M/L/X</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>50, 100</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>AdamW</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>validated + selected internal test</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Prepared next run</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>60:20:20</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>YOLOv12N/S/M/L/X</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>50, 100</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>AdamW</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>dataset prepared; full grid training pending</t>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>validated full B16 E50/E100 grid + selected internal test</t>
         </is>
       </c>
     </row>
@@ -998,146 +1010,287 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Metric_Source</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Variant</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Epoch_Setting</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Batch</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Recall</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>mAP50</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>mAP50-95</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Validation best</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>80:10:10</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>YOLOV12N</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="4" t="n">
         <v>0.70309</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="4" t="n">
         <v>0.72859</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="4" t="n">
         <v>0.7156129066551185</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="4" t="n">
         <v>0.7912400000000001</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="4" t="n">
         <v>0.39298</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Best by validation mAP50</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Internal test</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80:10:10</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>YOLOV12N</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="4" t="n">
         <v>0.5974608434168509</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="4" t="n">
         <v>0.6406926406926406</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="4" t="n">
         <v>0.6183219938269687</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="4" t="n">
         <v>0.7551453513733671</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="4" t="n">
         <v>0.4258796257028965</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Test using best validation model</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Best_Validation_Model</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Best_Val_Epoch</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Validation_mAP50</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Validation_F1</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Internal_Test_mAP50</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Internal_Test_F1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>80:10:10</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>YOLOV12N E50 B16</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0.7912400000000001</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0.7156129066551185</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0.7551453513733671</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0.6183219938269687</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>70:15:15</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>YOLOV12L E100 B16</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.7754799999999999</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.7076937839288236</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.6015102187896298</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.6010491916316369</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>60:20:20</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>YOLOV12S E100 B16</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.73873</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.676525715799154</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.6605311229283004</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0.620274837959925</v>
       </c>
     </row>
   </sheetData>

</xml_diff>